<commit_message>
Update energy matching and settlement handling
</commit_message>
<xml_diff>
--- a/server/source-templates/consumption-template.xlsx
+++ b/server/source-templates/consumption-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stefani/Desktop/MSIN0114/Utilidex/Dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33414D2B-D7E6-A648-8091-4765288E5A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ECB7855-18E9-354C-B91C-A851A58AF7F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16900" xr2:uid="{78BF5E39-7BDE-1448-A361-654C4F0EFA65}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Site ID</t>
   </si>
@@ -51,6 +51,12 @@
   </si>
   <si>
     <t>Date (dd/mm/yyyy)</t>
+  </si>
+  <si>
+    <t>Clock Change Period 1</t>
+  </si>
+  <si>
+    <t>Clock Change Period 2</t>
   </si>
 </sst>
 </file>
@@ -430,13 +436,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9FE031D-5A2C-AB4D-BF89-6D183D895C6A}">
-  <dimension ref="A1:AZ1"/>
+  <dimension ref="A1:BB1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="52" max="53" width="19.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" ht="17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:54" ht="17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -591,6 +598,12 @@
         <v>0</v>
       </c>
       <c r="AZ1" t="s">
+        <v>4</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>5</v>
+      </c>
+      <c r="BB1" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>